<commit_message>
Feat: Import bank statements that have no pay order no or txn ref
- Only Value Date is required; rows without a key are identified by content, slip number (Narration 1) and CNIC (Narrations 2-5)
- Duplicates of key-less rows are flagged (already in database, repeated in file, possible duplicate) and imported unless the user ticks Skip flagged duplicates
- Rows with a full key keep Conflict / Overwrite; Query pages, sorts and exports by Id and gains a Slip no filter and a CNIC filter that also finds narration CNICs
- Tests rewritten for the new rule plus key-less contract, upgrade and extractor tests; synthetic statement samples added

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Samples/test/05_missing_required_header.xlsx
+++ b/Samples/test/05_missing_required_header.xlsx
@@ -16,10 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
       <name val="Calibri"/>
@@ -49,9 +46,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -452,57 +448,57 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Value Date</t>
+          <t>Br. Code</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Br. Code</t>
+          <t>Branch Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Branch Name</t>
+          <t>Reg No</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Reg No</t>
+          <t>Application No</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Application No</t>
+          <t>Plot No</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Plot No</t>
+          <t>Street No</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Street No</t>
+          <t>Challan No</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Challan No</t>
+          <t>Customer Name</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Customer Name</t>
+          <t>Cheque/Inst No</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Cheque/Inst No</t>
+          <t>CNIC No</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>CNIC No</t>
+          <t>payorder no</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -587,27 +583,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
-        <v>45384</v>
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>0202</t>
+        </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>0202</t>
+          <t>Saddar Branch</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Saddar Branch</t>
+          <t>00001</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>00001</t>
+          <t>APP-E0001</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>APP-E0001</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -617,27 +615,27 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>CH985323</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>CH985323</t>
+          <t>Sara Malik</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Sara Malik</t>
+          <t>6023347</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>6023347</t>
+          <t>35202-5706031-6</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>35202-5706031-6</t>
+          <t>PO-E-0001</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -697,27 +695,29 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
-        <v>45385</v>
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>0303</t>
+        </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>0303</t>
+          <t>DHA Branch</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>DHA Branch</t>
+          <t>00002</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>00002</t>
+          <t>APP-E0002</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>APP-E0002</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -727,27 +727,27 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>CH933631</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>CH933631</t>
+          <t>Bilal Hussain</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Bilal Hussain</t>
+          <t>9950941</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>9950941</t>
+          <t>35202-6877482-1</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>35202-6877482-1</t>
+          <t>PO-E-0002</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
@@ -807,27 +807,29 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
-        <v>45386</v>
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>0404</t>
+        </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>0404</t>
+          <t>Gulshan Branch</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Gulshan Branch</t>
+          <t>00003</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>00003</t>
+          <t>APP-E0003</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>APP-E0003</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
@@ -837,27 +839,27 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>CH780915</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>CH780915</t>
+          <t>Ayesha Siddiqui</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Ayesha Siddiqui</t>
+          <t>2664337</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2664337</t>
+          <t>35202-6593387-9</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>35202-6593387-9</t>
+          <t>PO-E-0003</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
@@ -917,27 +919,29 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="n">
-        <v>45387</v>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>0101</t>
+          <t>Clifton Branch</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Clifton Branch</t>
+          <t>00004</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>00004</t>
+          <t>APP-E0004</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>APP-E0004</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -947,27 +951,27 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>CH120882</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>CH120882</t>
+          <t>Usman Tariq</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Usman Tariq</t>
+          <t>5967306</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>5967306</t>
+          <t>35202-5704469-3</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>35202-5704469-3</t>
+          <t>PO-E-0004</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
@@ -1027,27 +1031,29 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="1" t="n">
-        <v>45388</v>
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>0202</t>
+        </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>0202</t>
+          <t>Saddar Branch</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Saddar Branch</t>
+          <t>00005</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>00005</t>
+          <t>APP-E0005</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>APP-E0005</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -1057,27 +1063,27 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>CH908618</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>CH908618</t>
+          <t>Fatima Noor</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Fatima Noor</t>
+          <t>9822136</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>9822136</t>
+          <t>35202-5545315-1</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>35202-5545315-1</t>
+          <t>PO-E-0005</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
@@ -1137,27 +1143,29 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>45389</v>
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>0303</t>
+        </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>0303</t>
+          <t>DHA Branch</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DHA Branch</t>
+          <t>00006</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>00006</t>
+          <t>APP-E0006</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>APP-E0006</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -1167,27 +1175,27 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>CH962248</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>CH962248</t>
+          <t>Hamza Qureshi</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Hamza Qureshi</t>
+          <t>6232873</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>6232873</t>
+          <t>35202-5137490-6</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>35202-5137490-6</t>
+          <t>PO-E-0006</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1247,27 +1255,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>45390</v>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>0404</t>
+        </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>0404</t>
+          <t>Gulshan Branch</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gulshan Branch</t>
+          <t>00007</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>00007</t>
+          <t>APP-E0007</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>APP-E0007</t>
+          <t>8</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -1277,27 +1287,27 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>CH942004</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>CH942004</t>
+          <t>Zainab Ali</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Zainab Ali</t>
+          <t>8182831</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>8182831</t>
+          <t>35202-7753001-6</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>35202-7753001-6</t>
+          <t>PO-E-0007</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
@@ -1357,27 +1367,29 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>45391</v>
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>0101</t>
+        </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>0101</t>
+          <t>Clifton Branch</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Clifton Branch</t>
+          <t>00008</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>00008</t>
+          <t>APP-E0008</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>APP-E0008</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -1387,27 +1399,27 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>CH739248</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>CH739248</t>
+          <t>Imran Sheikh</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Imran Sheikh</t>
+          <t>6293274</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>6293274</t>
+          <t>35202-8027683-1</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>35202-8027683-1</t>
+          <t>PO-E-0008</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
@@ -1467,27 +1479,29 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>45392</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>0202</t>
+        </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>0202</t>
+          <t>Saddar Branch</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Saddar Branch</t>
+          <t>00009</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>00009</t>
+          <t>APP-E0009</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>APP-E0009</t>
+          <t>10</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -1497,27 +1511,27 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>CH963972</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>CH963972</t>
+          <t>Hina Raza</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Hina Raza</t>
+          <t>9483914</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>9483914</t>
+          <t>35202-2885174-9</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>35202-2885174-9</t>
+          <t>PO-E-0009</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
@@ -1577,27 +1591,29 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="n">
-        <v>45393</v>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>0303</t>
+        </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0303</t>
+          <t>DHA Branch</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>DHA Branch</t>
+          <t>00010</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>00010</t>
+          <t>APP-E0010</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>APP-E0010</t>
+          <t>11</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
@@ -1607,27 +1623,27 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>CH455614</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>CH455614</t>
+          <t>Kamran Butt</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Kamran Butt</t>
+          <t>5198225</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>5198225</t>
+          <t>35202-9120765-4</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>35202-9120765-4</t>
+          <t>PO-E-0010</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">

</xml_diff>